<commit_message>
Atualiza notas 3D Manha 2º Bimestre e adiciona .gitignore
</commit_message>
<xml_diff>
--- a/sources/3D_Manha_2_Bimestre.xlsx
+++ b/sources/3D_Manha_2_Bimestre.xlsx
@@ -61,7 +61,7 @@
     <x:t>Conselho Segundo Bimestre</x:t>
   </x:si>
   <x:si>
-    <x:t>267</x:t>
+    <x:t>317</x:t>
   </x:si>
   <x:si>
     <x:t>0 (Soma de todas as eletivas)</x:t>
@@ -207,7 +207,7 @@
     <x:t>64%</x:t>
   </x:si>
   <x:si>
-    <x:t>70%</x:t>
+    <x:t>69%</x:t>
   </x:si>
   <x:si>
     <x:t>ARTHUR ANTONIO SANTOS PIRES</x:t>
@@ -222,276 +222,288 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
+    <x:t>13</x:t>
+  </x:si>
+  <x:si>
     <x:t>9</x:t>
   </x:si>
   <x:si>
+    <x:t>84%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>82%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVELINO LOPES MABIALA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>88%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>91%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DANIEL QUENTA ARUQUIPA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>77%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>80%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDER DA SILVA CAMPOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>85%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GABRIELA SANTIAGO CONDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Não Comparecimento</x:t>
+  </x:si>
+  <x:si>
+    <x:t>16</x:t>
+  </x:si>
+  <x:si>
+    <x:t>75%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>66%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEOVANNA SILVA CESARIO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>76%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUILHERME PERRUCIO ANDRADE DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>89%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HIAGO DOS SANTOS ALVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>24</x:t>
+  </x:si>
+  <x:si>
+    <x:t>58%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>68%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INES MARIA CAMALANDUA MAYOMBE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>93%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISABELLA BARROS RODRIGUES DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Transferido</x:t>
+  </x:si>
+  <x:si>
+    <x:t>96%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISAQUE DE ALMEIDA SOUZA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>78%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>83%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISMAEL ARAO DE SOUZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JULIA SANTANA DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>100%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>99%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAIQUE CARVALHO GHIDINI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>79%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAUAN SAMUEL GONÇALVES SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>19</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAUAN VINICIUS CREPALDI RAMOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LAIS RAQUELLI PEREIRA DE LIMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LEONARDO FERNANDES BOSAK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>23</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>61%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUCAS DE SOUSA FERREIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>32</x:t>
+  </x:si>
+  <x:si>
+    <x:t>26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>56%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>98%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUIGI DE OLIVEIRA FRANCELINO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUIZA LIMA FERNANDES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>87%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARIA VITÓRIA SOARES RODRIGUES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>73%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MATHEUS DOS SANTOS GENIAL LIMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Remanejamento</x:t>
+  </x:si>
+  <x:si>
     <x:t>86%</x:t>
   </x:si>
   <x:si>
-    <x:t>83%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVELINO LOPES MABIALA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>88%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>91%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DANIEL QUENTA ARUQUIPA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>76%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>79%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EDER DA SILVA CAMPOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>87%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>85%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GABRIELA SANTIAGO CONDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Não Comparecimento</x:t>
-  </x:si>
-  <x:si>
-    <x:t>16</x:t>
-  </x:si>
-  <x:si>
-    <x:t>63%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEOVANNA SILVA CESARIO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>82%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUILHERME PERRUCIO ANDRADE DA SILVA</x:t>
+    <x:t>MATHEUS SALES DE OLIVEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MICAELI MONTEIRO OLIVEIRA SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MIGUEL AUGUSTO FERNANDES LEITE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NATHALIA SANTANA MONTEIRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NICOLE MONTEIRO DO CARMO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NICOLLY MARIANA VALDEVINO CARDOSO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>67%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEDRO PORTINHO FREITAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAFAEL MONTEIRO SOUSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>74%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RICARDO HENRIQUE DE CASTRO GALLO PONTES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ROBERTA DOS SANTOS ALCANTARA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VALDEMIRO JOSÉ DA COSTA CASSUA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>94%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VITOR HUGO OLIVEIRA MARIANO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>97%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VITOR SOUZA SANTOS SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>81%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VITÓRIA HELENA SANTOS DO NASCIMENTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>72%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WELLINTON CAUÃ SILVA COSTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WESLLEY JORGE RODRIGUES DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YAN NICACIO NASCIMENTO</x:t>
   </x:si>
   <x:si>
     <x:t>90%</x:t>
   </x:si>
   <x:si>
-    <x:t>89%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HIAGO DOS SANTOS ALVES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>59%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INES MARIA CAMALANDUA MAYOMBE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>93%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISABELLA BARROS RODRIGUES DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Transferido</x:t>
+    <x:t>YASMIM FERNANDES FELIX</x:t>
   </x:si>
   <x:si>
     <x:t>95%</x:t>
   </x:si>
   <x:si>
-    <x:t>ISAQUE DE ALMEIDA SOUZA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISMAEL ARAO DE SOUZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>80%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JULIA SANTANA DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>100%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>99%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAIQUE CARVALHO GHIDINI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>81%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>84%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAUAN SAMUEL GONÇALVES SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>71%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>77%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAUAN VINICIUS CREPALDI RAMOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>96%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LAIS RAQUELLI PEREIRA DE LIMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>75%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LEONARDO FERNANDES BOSAK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>23</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22</x:t>
+    <x:t>YASMIM HELENA SANTOS DO NASCIMENTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WILDER MAMANI VENTURA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JOAO VICTOR CAVALCANTI MACHADO</x:t>
   </x:si>
   <x:si>
     <x:t>62%</x:t>
   </x:si>
   <x:si>
-    <x:t>LUCAS DE SOUSA FERREIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>32</x:t>
-  </x:si>
-  <x:si>
-    <x:t>56%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUIGI DE OLIVEIRA FRANCELINO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUIZA LIMA FERNANDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARIA VITÓRIA SOARES RODRIGUES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MATHEUS DOS SANTOS GENIAL LIMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Remanejamento</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MATHEUS SALES DE OLIVEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>58%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>69%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MICAELI MONTEIRO OLIVEIRA SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MIGUEL AUGUSTO FERNANDES LEITE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NATHALIA SANTANA MONTEIRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NICOLE MONTEIRO DO CARMO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NICOLLY MARIANA VALDEVINO CARDOSO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>68%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEDRO PORTINHO FREITAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>73%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAFAEL MONTEIRO SOUSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RICARDO HENRIQUE DE CASTRO GALLO PONTES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ROBERTA DOS SANTOS ALCANTARA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VALDEMIRO JOSÉ DA COSTA CASSUA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>94%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VITOR HUGO OLIVEIRA MARIANO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>97%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VITOR SOUZA SANTOS SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VITÓRIA HELENA SANTOS DO NASCIMENTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WELLINTON CAUÃ SILVA COSTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WESLLEY JORGE RODRIGUES DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>78%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YAN NICACIO NASCIMENTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>92%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YASMIM FERNANDES FELIX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YASMIM HELENA SANTOS DO NASCIMENTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>74%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WILDER MAMANI VENTURA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JOAO VICTOR CAVALCANTI MACHADO</x:t>
-  </x:si>
-  <x:si>
     <x:t>CARLOS DANIEL TEIXEIRA DA SILVA</x:t>
   </x:si>
   <x:si>
@@ -504,9 +516,6 @@
     <x:t>MURILO DAMASCENO DAS NEVES</x:t>
   </x:si>
   <x:si>
-    <x:t>98%</x:t>
-  </x:si>
-  <x:si>
     <x:t>LETICIA LOHANNY MARQUES TAVARES</x:t>
   </x:si>
   <x:si>
@@ -529,6 +538,9 @@
   </x:si>
   <x:si>
     <x:t>Aulas Dadas: 48</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Aulas Dadas: 50</x:t>
   </x:si>
   <x:si>
     <x:t>Aulas Dadas: 34</x:t>
@@ -1581,13 +1593,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AN13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ13" s="12">
         <x:v>1</x:v>
@@ -1638,13 +1650,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG13" s="12">
-        <x:v>95</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="BH13" s="12" t="s">
         <x:v>58</x:v>
       </x:c>
       <x:c r="BI13" s="12">
-        <x:v>181</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="BJ13" s="12" t="s">
         <x:v>59</x:v>
@@ -1769,13 +1781,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AN14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="AP14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ14" s="12">
         <x:v>2</x:v>
@@ -1817,7 +1829,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="BD14" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BE14" s="12" t="s">
         <x:v>49</x:v>
@@ -1826,21 +1838,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG14" s="12">
-        <x:v>37</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="BH14" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="BI14" s="12">
-        <x:v>101</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="BJ14" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:62">
       <x:c r="A15" s="11" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B15" s="12" t="s">
         <x:v>47</x:v>
@@ -1861,7 +1873,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="H15" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="I15" s="12" t="s">
         <x:v>54</x:v>
@@ -1873,7 +1885,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="L15" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M15" s="12" t="s">
         <x:v>61</x:v>
@@ -1897,7 +1909,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="T15" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="U15" s="12" t="s">
         <x:v>61</x:v>
@@ -1957,13 +1969,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AN15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AO15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AP15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ15" s="12">
         <x:v>3</x:v>
@@ -2005,7 +2017,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="BD15" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BE15" s="12" t="s">
         <x:v>49</x:v>
@@ -2014,21 +2026,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG15" s="12">
-        <x:v>33</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="BH15" s="12" t="s">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="BI15" s="12">
-        <x:v>55</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="BJ15" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:62">
       <x:c r="A16" s="11" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B16" s="12" t="s">
         <x:v>47</x:v>
@@ -2124,7 +2136,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AG16" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AH16" s="12" t="s">
         <x:v>48</x:v>
@@ -2145,13 +2157,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AN16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AP16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ16" s="12">
         <x:v>4</x:v>
@@ -2202,21 +2214,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG16" s="12">
-        <x:v>65</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="BH16" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="BI16" s="12">
-        <x:v>123</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="BJ16" s="12" t="s">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:62">
       <x:c r="A17" s="11" t="s">
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B17" s="12" t="s">
         <x:v>47</x:v>
@@ -2333,13 +2345,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="AN17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AP17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ17" s="12">
         <x:v>5</x:v>
@@ -2390,13 +2402,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG17" s="12">
-        <x:v>36</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="BH17" s="12" t="s">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="BI17" s="12">
-        <x:v>89</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="BJ17" s="12" t="s">
         <x:v>76</x:v>
@@ -2524,10 +2536,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO18" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP18" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ18" s="12">
         <x:v>6</x:v>
@@ -2581,18 +2593,18 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="BH18" s="12" t="s">
-        <x:v>59</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="BI18" s="12">
         <x:v>215</x:v>
       </x:c>
       <x:c r="BJ18" s="12" t="s">
-        <x:v>80</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:62">
       <x:c r="A19" s="11" t="s">
-        <x:v>81</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B19" s="12" t="s">
         <x:v>47</x:v>
@@ -2709,13 +2721,13 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="AN19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="AP19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ19" s="12">
         <x:v>7</x:v>
@@ -2766,21 +2778,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG19" s="12">
-        <x:v>64</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="BH19" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="BI19" s="12">
-        <x:v>106</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="BJ19" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:62">
       <x:c r="A20" s="11" t="s">
-        <x:v>83</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B20" s="12" t="s">
         <x:v>47</x:v>
@@ -2897,13 +2909,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="AN20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ20" s="12">
         <x:v>8</x:v>
@@ -2954,13 +2966,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG20" s="12">
-        <x:v>28</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="BH20" s="12" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="BI20" s="12">
-        <x:v>65</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="BJ20" s="12" t="s">
         <x:v>85</x:v>
@@ -2980,7 +2992,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="E21" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F21" s="12" t="s">
         <x:v>49</x:v>
@@ -3052,7 +3064,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="AC21" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AD21" s="12" t="s">
         <x:v>49</x:v>
@@ -3085,13 +3097,13 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="AN21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AP21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ21" s="12">
         <x:v>9</x:v>
@@ -3100,7 +3112,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AS21" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AT21" s="12" t="s">
         <x:v>49</x:v>
@@ -3142,21 +3154,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG21" s="12">
-        <x:v>109</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="BH21" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="BI21" s="12">
-        <x:v>181</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="BJ21" s="12" t="s">
-        <x:v>59</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:62">
       <x:c r="A22" s="11" t="s">
-        <x:v>88</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B22" s="12" t="s">
         <x:v>47</x:v>
@@ -3165,7 +3177,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="D22" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E22" s="12" t="s">
         <x:v>49</x:v>
@@ -3189,7 +3201,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="L22" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M22" s="12" t="s">
         <x:v>50</x:v>
@@ -3273,13 +3285,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="AN22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AO22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AP22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ22" s="12">
         <x:v>10</x:v>
@@ -3330,24 +3342,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG22" s="12">
-        <x:v>25</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="BH22" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="BI22" s="12">
-        <x:v>43</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="BJ22" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:62">
       <x:c r="A23" s="11" t="s">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B23" s="12" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C23" s="12">
         <x:v>11</x:v>
@@ -3464,10 +3476,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ23" s="12">
         <x:v>11</x:v>
@@ -3521,7 +3533,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="BH23" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="BI23" s="12">
         <x:v>99</x:v>
@@ -3532,7 +3544,7 @@
     </x:row>
     <x:row r="24" spans="1:62">
       <x:c r="A24" s="11" t="s">
-        <x:v>93</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B24" s="12" t="s">
         <x:v>47</x:v>
@@ -3640,7 +3652,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AK24" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AL24" s="12" t="s">
         <x:v>49</x:v>
@@ -3649,13 +3661,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="AN24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ24" s="12">
         <x:v>12</x:v>
@@ -3706,21 +3718,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG24" s="12">
-        <x:v>65</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="BH24" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="BI24" s="12">
-        <x:v>103</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="BJ24" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:62">
       <x:c r="A25" s="11" t="s">
-        <x:v>94</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B25" s="12" t="s">
         <x:v>47</x:v>
@@ -3795,7 +3807,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="Z25" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="AA25" s="12">
         <x:v>13</x:v>
@@ -3837,13 +3849,13 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="AN25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AP25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ25" s="12">
         <x:v>13</x:v>
@@ -3894,24 +3906,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG25" s="12">
-        <x:v>54</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="BH25" s="12" t="s">
-        <x:v>96</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="BI25" s="12">
-        <x:v>101</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="BJ25" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:62">
       <x:c r="A26" s="11" t="s">
-        <x:v>97</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B26" s="12" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C26" s="12">
         <x:v>14</x:v>
@@ -4028,10 +4040,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ26" s="12">
         <x:v>14</x:v>
@@ -4085,18 +4097,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH26" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BI26" s="12">
         <x:v>6</x:v>
       </x:c>
       <x:c r="BJ26" s="12" t="s">
-        <x:v>99</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:62">
       <x:c r="A27" s="11" t="s">
-        <x:v>100</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B27" s="12" t="s">
         <x:v>47</x:v>
@@ -4213,13 +4225,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="AN27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="AP27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ27" s="12">
         <x:v>15</x:v>
@@ -4270,21 +4282,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG27" s="12">
-        <x:v>52</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BH27" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="BI27" s="12">
-        <x:v>94</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="BJ27" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:62">
       <x:c r="A28" s="11" t="s">
-        <x:v>103</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B28" s="12" t="s">
         <x:v>47</x:v>
@@ -4401,13 +4413,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="AN28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="AP28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ28" s="12">
         <x:v>16</x:v>
@@ -4458,21 +4470,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG28" s="12">
-        <x:v>78</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH28" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="BI28" s="12">
-        <x:v>135</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="BJ28" s="12" t="s">
-        <x:v>105</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:62">
       <x:c r="A29" s="11" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B29" s="12" t="s">
         <x:v>47</x:v>
@@ -4481,7 +4493,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="D29" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E29" s="12" t="s">
         <x:v>49</x:v>
@@ -4505,7 +4517,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="L29" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M29" s="12" t="s">
         <x:v>61</x:v>
@@ -4529,7 +4541,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="T29" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="U29" s="12" t="s">
         <x:v>63</x:v>
@@ -4553,7 +4565,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="AB29" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC29" s="12" t="s">
         <x:v>63</x:v>
@@ -4589,13 +4601,13 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="AN29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AP29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ29" s="12">
         <x:v>17</x:v>
@@ -4646,21 +4658,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG29" s="12">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="BH29" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="BI29" s="12">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="BJ29" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:62">
       <x:c r="A30" s="11" t="s">
-        <x:v>108</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B30" s="12" t="s">
         <x:v>47</x:v>
@@ -4777,13 +4789,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="AN30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AP30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ30" s="12">
         <x:v>18</x:v>
@@ -4834,16 +4846,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG30" s="12">
-        <x:v>66</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="BH30" s="12" t="s">
-        <x:v>109</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="BI30" s="12">
-        <x:v>146</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="BJ30" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:62">
@@ -4965,13 +4977,13 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="AN31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AP31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AQ31" s="12">
         <x:v>19</x:v>
@@ -5019,19 +5031,19 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="BF31" s="12" t="s">
-        <x:v>49</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BG31" s="12">
-        <x:v>101</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="BH31" s="12" t="s">
         <x:v>113</x:v>
       </x:c>
       <x:c r="BI31" s="12">
-        <x:v>60</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="BJ31" s="12" t="s">
-        <x:v>84</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:62">
@@ -5072,7 +5084,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="M32" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N32" s="12" t="s">
         <x:v>49</x:v>
@@ -5120,7 +5132,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AC32" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="AD32" s="12" t="s">
         <x:v>49</x:v>
@@ -5135,7 +5147,7 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="AH32" s="12" t="s">
-        <x:v>115</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AI32" s="12">
         <x:v>20</x:v>
@@ -5144,22 +5156,22 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="AK32" s="12" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AL32" s="12" t="s">
-        <x:v>116</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="AM32" s="12">
         <x:v>20</x:v>
       </x:c>
       <x:c r="AN32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="AP32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="AQ32" s="12">
         <x:v>20</x:v>
@@ -5204,27 +5216,27 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="BE32" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BF32" s="12" t="s">
-        <x:v>49</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="BG32" s="12">
-        <x:v>118</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="BH32" s="12" t="s">
         <x:v>117</x:v>
       </x:c>
       <x:c r="BI32" s="12">
-        <x:v>42</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="BJ32" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:62">
       <x:c r="A33" s="11" t="s">
-        <x:v>118</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B33" s="12" t="s">
         <x:v>47</x:v>
@@ -5317,7 +5329,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="AF33" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AG33" s="12" t="s">
         <x:v>49</x:v>
@@ -5341,13 +5353,13 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="AN33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AO33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ33" s="12">
         <x:v>21</x:v>
@@ -5401,18 +5413,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH33" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BI33" s="12">
         <x:v>-2</x:v>
       </x:c>
       <x:c r="BJ33" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:62">
       <x:c r="A34" s="11" t="s">
-        <x:v>119</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B34" s="12" t="s">
         <x:v>47</x:v>
@@ -5445,7 +5457,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="L34" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M34" s="12" t="s">
         <x:v>63</x:v>
@@ -5529,13 +5541,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="AN34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AO34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AP34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ34" s="12">
         <x:v>22</x:v>
@@ -5577,7 +5589,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="BD34" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BE34" s="12" t="s">
         <x:v>61</x:v>
@@ -5586,13 +5598,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG34" s="12">
-        <x:v>33</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="BH34" s="12" t="s">
-        <x:v>68</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="BI34" s="12">
-        <x:v>67</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="BJ34" s="12" t="s">
         <x:v>85</x:v>
@@ -5600,7 +5612,7 @@
     </x:row>
     <x:row r="35" spans="1:62">
       <x:c r="A35" s="11" t="s">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B35" s="12" t="s">
         <x:v>78</x:v>
@@ -5720,10 +5732,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ35" s="12">
         <x:v>23</x:v>
@@ -5777,21 +5789,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH35" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BI35" s="12">
         <x:v>168</x:v>
       </x:c>
       <x:c r="BJ35" s="12" t="s">
-        <x:v>104</x:v>
+        <x:v>123</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:62">
       <x:c r="A36" s="11" t="s">
-        <x:v>121</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B36" s="12" t="s">
-        <x:v>122</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="C36" s="12">
         <x:v>24</x:v>
@@ -5908,10 +5920,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ36" s="12">
         <x:v>24</x:v>
@@ -5965,18 +5977,18 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="BH36" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="BI36" s="12">
         <x:v>89</x:v>
       </x:c>
       <x:c r="BJ36" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:62">
       <x:c r="A37" s="11" t="s">
-        <x:v>123</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B37" s="12" t="s">
         <x:v>47</x:v>
@@ -6060,7 +6072,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AC37" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AD37" s="12" t="s">
         <x:v>49</x:v>
@@ -6072,7 +6084,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AG37" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="AH37" s="12" t="s">
         <x:v>49</x:v>
@@ -6084,7 +6096,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AK37" s="12" t="s">
-        <x:v>115</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AL37" s="12" t="s">
         <x:v>49</x:v>
@@ -6093,13 +6105,13 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="AN37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="AP37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ37" s="12">
         <x:v>25</x:v>
@@ -6123,7 +6135,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AX37" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AY37" s="12">
         <x:v>25</x:v>
@@ -6150,21 +6162,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG37" s="12">
-        <x:v>111</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="BH37" s="12" t="s">
-        <x:v>124</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="BI37" s="12">
-        <x:v>183</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="BJ37" s="12" t="s">
-        <x:v>125</x:v>
+        <x:v>89</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:62">
       <x:c r="A38" s="11" t="s">
-        <x:v>126</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B38" s="12" t="s">
         <x:v>47</x:v>
@@ -6281,13 +6293,13 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="AN38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AO38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ38" s="12">
         <x:v>26</x:v>
@@ -6338,13 +6350,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG38" s="12">
-        <x:v>61</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BH38" s="12" t="s">
-        <x:v>105</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="BI38" s="12">
-        <x:v>122</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="BJ38" s="12" t="s">
         <x:v>96</x:v>
@@ -6352,7 +6364,7 @@
     </x:row>
     <x:row r="39" spans="1:62">
       <x:c r="A39" s="11" t="s">
-        <x:v>127</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B39" s="12" t="s">
         <x:v>47</x:v>
@@ -6469,13 +6481,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="AN39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ39" s="12">
         <x:v>27</x:v>
@@ -6526,21 +6538,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG39" s="12">
-        <x:v>29</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="BH39" s="12" t="s">
         <x:v>85</x:v>
       </x:c>
       <x:c r="BI39" s="12">
-        <x:v>80</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="BJ39" s="12" t="s">
-        <x:v>75</x:v>
+        <x:v>121</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:62">
       <x:c r="A40" s="11" t="s">
-        <x:v>128</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B40" s="12" t="s">
         <x:v>47</x:v>
@@ -6657,13 +6669,13 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="AN40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AP40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ40" s="12">
         <x:v>28</x:v>
@@ -6714,21 +6726,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG40" s="12">
-        <x:v>42</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="BH40" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI40" s="12">
-        <x:v>83</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="BJ40" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:62">
       <x:c r="A41" s="11" t="s">
-        <x:v>129</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B41" s="12" t="s">
         <x:v>47</x:v>
@@ -6785,7 +6797,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="T41" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="U41" s="12" t="s">
         <x:v>54</x:v>
@@ -6845,13 +6857,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="AN41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ41" s="12">
         <x:v>29</x:v>
@@ -6902,21 +6914,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG41" s="12">
-        <x:v>40</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="BH41" s="12" t="s">
         <x:v>76</x:v>
       </x:c>
       <x:c r="BI41" s="12">
-        <x:v>82</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="BJ41" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:62">
       <x:c r="A42" s="11" t="s">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B42" s="12" t="s">
         <x:v>47</x:v>
@@ -7000,7 +7012,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AC42" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AD42" s="12" t="s">
         <x:v>49</x:v>
@@ -7012,7 +7024,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AG42" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AH42" s="12" t="s">
         <x:v>49</x:v>
@@ -7033,13 +7045,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="AN42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="AP42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ42" s="12">
         <x:v>30</x:v>
@@ -7090,21 +7102,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG42" s="12">
-        <x:v>102</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="BH42" s="12" t="s">
         <x:v>113</x:v>
       </x:c>
       <x:c r="BI42" s="12">
-        <x:v>193</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="BJ42" s="12" t="s">
-        <x:v>131</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:62">
       <x:c r="A43" s="11" t="s">
-        <x:v>132</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B43" s="12" t="s">
         <x:v>47</x:v>
@@ -7200,7 +7212,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="AG43" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AH43" s="12" t="s">
         <x:v>49</x:v>
@@ -7212,7 +7224,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="AK43" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AL43" s="12" t="s">
         <x:v>49</x:v>
@@ -7221,13 +7233,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="AN43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="AP43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ43" s="12">
         <x:v>31</x:v>
@@ -7278,21 +7290,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG43" s="12">
-        <x:v>73</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BH43" s="12" t="s">
-        <x:v>133</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="BI43" s="12">
-        <x:v>107</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="BJ43" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:62">
       <x:c r="A44" s="11" t="s">
-        <x:v>134</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B44" s="12" t="s">
         <x:v>47</x:v>
@@ -7316,7 +7328,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="I44" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="J44" s="12" t="s">
         <x:v>49</x:v>
@@ -7400,7 +7412,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="AK44" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AL44" s="12" t="s">
         <x:v>49</x:v>
@@ -7409,13 +7421,13 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="AN44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AP44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ44" s="12">
         <x:v>32</x:v>
@@ -7466,21 +7478,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG44" s="12">
-        <x:v>71</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="BH44" s="12" t="s">
-        <x:v>133</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="BI44" s="12">
-        <x:v>93</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="BJ44" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:62">
       <x:c r="A45" s="11" t="s">
-        <x:v>135</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B45" s="12" t="s">
         <x:v>47</x:v>
@@ -7597,13 +7609,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AN45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ45" s="12">
         <x:v>33</x:v>
@@ -7654,13 +7666,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG45" s="12">
-        <x:v>37</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="BH45" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="BI45" s="12">
-        <x:v>91</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BJ45" s="12" t="s">
         <x:v>76</x:v>
@@ -7668,7 +7680,7 @@
     </x:row>
     <x:row r="46" spans="1:62">
       <x:c r="A46" s="11" t="s">
-        <x:v>136</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B46" s="12" t="s">
         <x:v>47</x:v>
@@ -7785,13 +7797,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="AN46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AP46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ46" s="12">
         <x:v>34</x:v>
@@ -7842,13 +7854,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG46" s="12">
-        <x:v>43</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="BH46" s="12" t="s">
-        <x:v>102</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI46" s="12">
-        <x:v>87</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="BJ46" s="12" t="s">
         <x:v>76</x:v>
@@ -7856,7 +7868,7 @@
     </x:row>
     <x:row r="47" spans="1:62">
       <x:c r="A47" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B47" s="12" t="s">
         <x:v>47</x:v>
@@ -7889,7 +7901,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="L47" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M47" s="12" t="s">
         <x:v>61</x:v>
@@ -7937,7 +7949,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="AB47" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC47" s="12" t="s">
         <x:v>61</x:v>
@@ -7961,7 +7973,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="AJ47" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AK47" s="12" t="s">
         <x:v>61</x:v>
@@ -7973,13 +7985,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="AN47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AO47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ47" s="12">
         <x:v>35</x:v>
@@ -8030,21 +8042,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG47" s="12">
-        <x:v>14</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="BH47" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="BI47" s="12">
-        <x:v>37</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="BJ47" s="12" t="s">
-        <x:v>138</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:62">
       <x:c r="A48" s="11" t="s">
-        <x:v>139</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B48" s="12" t="s">
         <x:v>47</x:v>
@@ -8137,7 +8149,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="AF48" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AG48" s="12" t="s">
         <x:v>54</x:v>
@@ -8161,13 +8173,13 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="AN48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AO48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AP48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ48" s="12">
         <x:v>36</x:v>
@@ -8218,21 +8230,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG48" s="12">
-        <x:v>19</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="BH48" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="BI48" s="12">
-        <x:v>18</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="BJ48" s="12" t="s">
-        <x:v>140</x:v>
+        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:62">
       <x:c r="A49" s="11" t="s">
-        <x:v>141</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B49" s="12" t="s">
         <x:v>47</x:v>
@@ -8349,13 +8361,13 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="AN49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AP49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ49" s="12">
         <x:v>37</x:v>
@@ -8397,7 +8409,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="BD49" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BE49" s="12" t="s">
         <x:v>54</x:v>
@@ -8406,21 +8418,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG49" s="12">
-        <x:v>49</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="BH49" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="BI49" s="12">
-        <x:v>112</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="BJ49" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>144</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:62">
       <x:c r="A50" s="11" t="s">
-        <x:v>142</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B50" s="12" t="s">
         <x:v>78</x:v>
@@ -8540,10 +8552,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ50" s="12">
         <x:v>38</x:v>
@@ -8597,18 +8609,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH50" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BI50" s="12">
         <x:v>173</x:v>
       </x:c>
       <x:c r="BJ50" s="12" t="s">
-        <x:v>59</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:62">
       <x:c r="A51" s="11" t="s">
-        <x:v>143</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B51" s="12" t="s">
         <x:v>47</x:v>
@@ -8725,13 +8737,13 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="AN51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="AP51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ51" s="12">
         <x:v>39</x:v>
@@ -8782,21 +8794,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG51" s="12">
-        <x:v>52</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BH51" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="BI51" s="12">
-        <x:v>122</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="BJ51" s="12" t="s">
-        <x:v>96</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:62">
       <x:c r="A52" s="11" t="s">
-        <x:v>144</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B52" s="12" t="s">
         <x:v>47</x:v>
@@ -8859,7 +8871,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="V52" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="W52" s="12">
         <x:v>40</x:v>
@@ -8907,19 +8919,19 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="AL52" s="12" t="s">
-        <x:v>145</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="AM52" s="12">
         <x:v>40</x:v>
       </x:c>
       <x:c r="AN52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AP52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="AQ52" s="12">
         <x:v>40</x:v>
@@ -8928,7 +8940,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AS52" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AT52" s="12" t="s">
         <x:v>79</x:v>
@@ -8967,24 +8979,24 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BF52" s="12" t="s">
-        <x:v>49</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BG52" s="12">
-        <x:v>59</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="BH52" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="BI52" s="12">
-        <x:v>17</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="BJ52" s="12" t="s">
-        <x:v>140</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:62">
       <x:c r="A53" s="11" t="s">
-        <x:v>147</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B53" s="12" t="s">
         <x:v>47</x:v>
@@ -9101,13 +9113,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="AN53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="AP53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ53" s="12">
         <x:v>41</x:v>
@@ -9158,21 +9170,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG53" s="12">
-        <x:v>19</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="BH53" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="BI53" s="12">
-        <x:v>50</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="BJ53" s="12" t="s">
-        <x:v>148</x:v>
+        <x:v>151</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:62">
       <x:c r="A54" s="11" t="s">
-        <x:v>149</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B54" s="12" t="s">
         <x:v>47</x:v>
@@ -9289,13 +9301,13 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="AN54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="AP54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ54" s="12">
         <x:v>42</x:v>
@@ -9346,21 +9358,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG54" s="12">
-        <x:v>7</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="BH54" s="12" t="s">
-        <x:v>140</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="BI54" s="12">
-        <x:v>37</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="BJ54" s="12" t="s">
-        <x:v>138</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:62">
       <x:c r="A55" s="11" t="s">
-        <x:v>150</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B55" s="12" t="s">
         <x:v>78</x:v>
@@ -9480,10 +9492,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ55" s="12">
         <x:v>43</x:v>
@@ -9537,18 +9549,18 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH55" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BI55" s="12">
         <x:v>148</x:v>
       </x:c>
       <x:c r="BJ55" s="12" t="s">
-        <x:v>151</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:62">
       <x:c r="A56" s="11" t="s">
-        <x:v>152</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B56" s="12" t="s">
         <x:v>47</x:v>
@@ -9656,7 +9668,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AK56" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AL56" s="12" t="s">
         <x:v>49</x:v>
@@ -9665,13 +9677,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="AN56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AP56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ56" s="12">
         <x:v>44</x:v>
@@ -9722,21 +9734,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG56" s="12">
-        <x:v>47</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="BH56" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BI56" s="12">
-        <x:v>52</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="BJ56" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:62">
       <x:c r="A57" s="11" t="s">
-        <x:v>153</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B57" s="12" t="s">
         <x:v>47</x:v>
@@ -9853,13 +9865,13 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="AN57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AO57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="AP57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ57" s="12">
         <x:v>45</x:v>
@@ -9910,21 +9922,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG57" s="12">
-        <x:v>100</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="BH57" s="12" t="s">
-        <x:v>80</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="BI57" s="12">
-        <x:v>110</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="BJ57" s="12" t="s">
-        <x:v>82</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:62">
       <x:c r="A58" s="11" t="s">
-        <x:v>154</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B58" s="12" t="s">
         <x:v>78</x:v>
@@ -10032,7 +10044,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK58" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AL58" s="12" t="s">
         <x:v>49</x:v>
@@ -10044,10 +10056,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ58" s="12">
         <x:v>46</x:v>
@@ -10101,18 +10113,18 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="BH58" s="12" t="s">
-        <x:v>151</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="BI58" s="12">
         <x:v>77</x:v>
       </x:c>
       <x:c r="BJ58" s="12" t="s">
-        <x:v>75</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:62">
       <x:c r="A59" s="11" t="s">
-        <x:v>155</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B59" s="12" t="s">
         <x:v>47</x:v>
@@ -10229,13 +10241,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="AN59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AO59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="AP59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ59" s="12">
         <x:v>47</x:v>
@@ -10286,21 +10298,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG59" s="12">
-        <x:v>23</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="BH59" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="BI59" s="12">
-        <x:v>21</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="BJ59" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>153</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:62">
       <x:c r="A60" s="11" t="s">
-        <x:v>156</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B60" s="12" t="s">
         <x:v>47</x:v>
@@ -10381,7 +10393,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AB60" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC60" s="12" t="s">
         <x:v>63</x:v>
@@ -10417,13 +10429,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AN60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AO60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AP60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ60" s="12">
         <x:v>48</x:v>
@@ -10474,24 +10486,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG60" s="12">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="BH60" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="BI60" s="12">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="BJ60" s="12" t="s">
-        <x:v>107</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:62">
       <x:c r="A61" s="11" t="s">
-        <x:v>157</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B61" s="12" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="C61" s="12">
         <x:v>49</x:v>
@@ -10608,10 +10620,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO61" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AP61" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ61" s="12">
         <x:v>49</x:v>
@@ -10665,18 +10677,18 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="BH61" s="12" t="s">
-        <x:v>158</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="BI61" s="12">
         <x:v>5</x:v>
       </x:c>
       <x:c r="BJ61" s="12" t="s">
-        <x:v>158</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:62">
       <x:c r="A62" s="11" t="s">
-        <x:v>159</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B62" s="12" t="s">
         <x:v>47</x:v>
@@ -10697,7 +10709,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="H62" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="I62" s="12" t="s">
         <x:v>49</x:v>
@@ -10793,13 +10805,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AN62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AP62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ62" s="12">
         <x:v>50</x:v>
@@ -10850,21 +10862,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG62" s="12">
-        <x:v>14</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="BH62" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="BI62" s="12">
-        <x:v>14</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="BJ62" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>140</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:62">
       <x:c r="A63" s="11" t="s">
-        <x:v>160</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B63" s="12" t="s">
         <x:v>47</x:v>
@@ -10981,13 +10993,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="AN63" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AO63" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AP63" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AQ63" s="12">
         <x:v>51</x:v>
@@ -11038,105 +11050,105 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG63" s="12">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="BH63" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="BI63" s="12">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="BJ63" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:62">
       <x:c r="A64" s="13" t="s">
-        <x:v>161</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B64" s="13" t="s">
-        <x:v>161</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C64" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D64" s="7"/>
       <x:c r="E64" s="7"/>
       <x:c r="F64" s="7"/>
       <x:c r="G64" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="H64" s="7"/>
       <x:c r="I64" s="7"/>
       <x:c r="J64" s="7"/>
       <x:c r="K64" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="L64" s="7"/>
       <x:c r="M64" s="7"/>
       <x:c r="N64" s="7"/>
       <x:c r="O64" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="P64" s="7"/>
       <x:c r="Q64" s="7"/>
       <x:c r="R64" s="7"/>
       <x:c r="S64" s="7" t="s">
-        <x:v>165</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="T64" s="7"/>
       <x:c r="U64" s="7"/>
       <x:c r="V64" s="7"/>
       <x:c r="W64" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="X64" s="7"/>
       <x:c r="Y64" s="7"/>
       <x:c r="Z64" s="7"/>
       <x:c r="AA64" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="AB64" s="7"/>
       <x:c r="AC64" s="7"/>
       <x:c r="AD64" s="7"/>
       <x:c r="AE64" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="AF64" s="7"/>
       <x:c r="AG64" s="7"/>
       <x:c r="AH64" s="7"/>
       <x:c r="AI64" s="7" t="s">
-        <x:v>166</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="AJ64" s="7"/>
       <x:c r="AK64" s="7"/>
       <x:c r="AL64" s="7"/>
       <x:c r="AM64" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="AN64" s="7"/>
       <x:c r="AO64" s="7"/>
       <x:c r="AP64" s="7"/>
       <x:c r="AQ64" s="7" t="s">
-        <x:v>167</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="AR64" s="7"/>
       <x:c r="AS64" s="7"/>
       <x:c r="AT64" s="7"/>
       <x:c r="AU64" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="AV64" s="7"/>
       <x:c r="AW64" s="7"/>
       <x:c r="AX64" s="7"/>
       <x:c r="AY64" s="7" t="s">
-        <x:v>168</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="AZ64" s="7"/>
       <x:c r="BA64" s="7"/>
       <x:c r="BB64" s="7"/>
       <x:c r="BC64" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="BD64" s="7"/>
       <x:c r="BE64" s="7"/>
@@ -11148,37 +11160,37 @@
     </x:row>
     <x:row r="66" spans="1:62">
       <x:c r="A66" s="14" t="s">
-        <x:v>169</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:62">
       <x:c r="A67" s="13" t="s">
-        <x:v>170</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:62">
       <x:c r="A68" s="13" t="s">
-        <x:v>171</x:v>
+        <x:v>175</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:62">
       <x:c r="A69" s="13" t="s">
-        <x:v>172</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:62">
       <x:c r="A70" s="13" t="s">
-        <x:v>173</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:62">
       <x:c r="A71" s="13" t="s">
-        <x:v>174</x:v>
+        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="72" spans="1:62">
       <x:c r="A72" s="13" t="s">
-        <x:v>175</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>